<commit_message>
added camera access video, test type mapping
</commit_message>
<xml_diff>
--- a/src/JET_Sample_Format.xlsx
+++ b/src/JET_Sample_Format.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Full Stack Development\Exam Portal\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A58AF87A-EAF3-4098-97B8-48B565CB6F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C13F6C4-DC06-46C2-87F8-E5259D5E46FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{FE836248-BE71-4985-A8D6-F5CC19AA9C75}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FE836248-BE71-4985-A8D6-F5CC19AA9C75}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
   <si>
     <t>Test Name</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>If you copy-paste text from word or internet, make sure to select paste values. Please do not change the formatting.</t>
+  </si>
+  <si>
+    <t>Exam Type</t>
   </si>
 </sst>
 </file>
@@ -517,15 +520,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -533,17 +539,17 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>50</v>
-      </c>
       <c r="D2">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E2">
-        <v>50</v>
+        <v>30</v>
+      </c>
+      <c r="F2">
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>